<commit_message>
Add AHSP reference mapping to analysis
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Analisa_Jam_Alat_dan_Kebutuhan_Material.xlsx
+++ b/Analisa_Jam_Alat_dan_Kebutuhan_Material.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Analisa_Jam_Alat" sheetId="7" r:id="rId7"/>
     <sheet name="Kebutuhan_Material" sheetId="8" r:id="rId8"/>
     <sheet name="Rekap" sheetId="9" r:id="rId9"/>
+    <sheet name="Referensi_AHSP" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -113,6 +114,416 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kode analisa</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Uraian pekerjaan</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kode AHSP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Alat/tenaga</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dasar perhitungan jam alat</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Halaman PDF</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>GRD</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Grading/perataan</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-GRD-PROV</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>AL-GRD</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>Luas / produktivitas grader</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>RIP</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Ripping/penggemburan</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-RIP-PROV</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>AL-DZR</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>Volume / Q dozer</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>SPR</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Spreading/penyebaran</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SPR-PROV</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>AL-DZR</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>Volume / Q dozer</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Compacting/pemadatan</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-CMP-PROV</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>AL-RLR + AL-WTR</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Volume / Q roller; air dihitung terpisah</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>DRN</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Drainase/galian</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>A.3.01.1a</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>AL-EXC</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Volume galian / Q excavator</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>Sekitar 324</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Perlu dicocokkan dengan PDF sumber</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>SUB</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Perbaikan tanah dasar</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SUB-PROV</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>AL-EXC</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>Volume / Q excavator</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>BSC</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Basecourse baru</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-BSC-PROV</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>AL-DZR + AL-RLR</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Volume basecourse / produktivitas pekerjaan</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>PTH</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Patching lubang</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-PTH-PROV</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>AL-EXC</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Volume patching / Q excavator</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>Semenisasi</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SEM-PROV</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Tenaga manual</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>Tidak ada jam alat berat pada model ini</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>Belum terverifikasi</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Kode internal sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Catatan penting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Nomor halaman resmi selain rujukan contoh galian belum diisi karena file PDF SE-DJBK No. 68/2024 Lampiran IV tidak tersedia di workspace saat workbook dibuat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Kode AHSP-SDA-*-PROV adalah kode internal analisa, bukan nomor item resmi. Ganti setelah PDF sumber dan edisi halaman dikonfirmasi.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:S52"/>
@@ -6703,7 +7114,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -6757,6 +7168,16 @@
           <t>Satuan koef.</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Kode AHSP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Halaman acuan</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -6795,6 +7216,16 @@
           <t>jam/m2</t>
         </is>
       </c>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-GRD-PROV</t>
+        </is>
+      </c>
+      <c r="J2" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -6833,6 +7264,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-RIP-PROV</t>
+        </is>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -6871,6 +7312,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I4" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SPR-PROV</t>
+        </is>
+      </c>
+      <c r="J4" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -6909,6 +7360,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-CMP-PROV</t>
+        </is>
+      </c>
+      <c r="J5" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -6947,6 +7408,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>A.3.01.1a</t>
+        </is>
+      </c>
+      <c r="J6" s="0" t="inlineStr">
+        <is>
+          <t>Sekitar hal. 324; verifikasi terhadap edisi PDF</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -6985,6 +7456,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SUB-PROV</t>
+        </is>
+      </c>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -7023,6 +7504,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-BSC-PROV</t>
+        </is>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -7061,6 +7552,16 @@
           <t>jam/m3</t>
         </is>
       </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-PTH-PROV</t>
+        </is>
+      </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -7097,6 +7598,16 @@
       <c r="H10" s="0" t="inlineStr">
         <is>
           <t>jam/m2</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>AHSP-SDA-SEM-PROV</t>
+        </is>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t>Lampiran IV; halaman belum terverifikasi</t>
         </is>
       </c>
     </row>

</xml_diff>